<commit_message>
optmized no learning familiarization stimuli
</commit_message>
<xml_diff>
--- a/stim/stim_list_no_learning_familiarization.xlsx
+++ b/stim/stim_list_no_learning_familiarization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\docs\code\matlab\Task_SpeechMotorSequenceLearning\stim\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Task\Task_SpeechMotorSequenceLearning\stim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268E2191-AB0C-4BF9-AD00-7379709E988C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16AEA9E0-DF48-4276-8701-36C2F7F3BE79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -610,7 +610,7 @@
         <v>2</v>
       </c>
       <c r="D14" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -638,7 +638,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>